<commit_message>
auto-publish rep recap: manual
</commit_message>
<xml_diff>
--- a/activity/WEEKLY_RECAP_REP.xlsx
+++ b/activity/WEEKLY_RECAP_REP.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2319" uniqueCount="558">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2583" uniqueCount="590">
   <si>
     <t>Weekly Rep Recap</t>
   </si>
@@ -1020,6 +1020,102 @@
   </si>
   <si>
     <t>New Clients — September 2026</t>
+  </si>
+  <si>
+    <t>New = customer's first invoice landed in this month · derived from invoice history through 2026-09-11</t>
+  </si>
+  <si>
+    <t>YTD New Clients</t>
+  </si>
+  <si>
+    <t>This Month</t>
+  </si>
+  <si>
+    <t>Last Month</t>
+  </si>
+  <si>
+    <t>Best Month (Apr)</t>
+  </si>
+  <si>
+    <t>Month-over-month · new clients by rep</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Karin</t>
+  </si>
+  <si>
+    <t>Megan</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>MoM Δ</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>+2</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>+6</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>+4</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>-8</t>
+  </si>
+  <si>
+    <t>June</t>
+  </si>
+  <si>
+    <t>-2</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>+1</t>
+  </si>
+  <si>
+    <t>August</t>
+  </si>
+  <si>
+    <t>+7</t>
+  </si>
+  <si>
+    <t>September (MTD)</t>
+  </si>
+  <si>
+    <t>-12</t>
+  </si>
+  <si>
+    <t>YTD Total</t>
+  </si>
+  <si>
+    <t>September new clients (2)</t>
+  </si>
+  <si>
+    <t>2026 new-client roster (75) — sorted newest first</t>
+  </si>
+  <si>
+    <t>First Invoice</t>
   </si>
   <si>
     <t>Outstanding Balances (Aging)</t>
@@ -1706,7 +1802,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0;(&quot;$&quot;#,##0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1848,6 +1944,34 @@
       <sz val="13"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="0C4E54"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="7A7974"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="1E7F3E"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="B22222"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1930,7 +2054,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -2073,6 +2197,33 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -3190,46 +3341,46 @@
         <v>262</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>338</v>
+        <v>370</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>339</v>
+        <v>371</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>224</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>340</v>
+        <v>372</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>341</v>
+        <v>373</v>
       </c>
       <c r="G1" s="9" t="s">
         <v>226</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>342</v>
+        <v>374</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>343</v>
+        <v>375</v>
       </c>
       <c r="J1" s="9" t="s">
         <v>227</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>344</v>
+        <v>376</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>345</v>
+        <v>377</v>
       </c>
       <c r="M1" s="9" t="s">
         <v>9</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>346</v>
+        <v>378</v>
       </c>
       <c r="O1" s="9" t="s">
-        <v>347</v>
+        <v>379</v>
       </c>
       <c r="P1" s="9" t="s">
         <v>229</v>
@@ -3240,10 +3391,10 @@
         <v>203</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>348</v>
+        <v>380</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>349</v>
+        <v>381</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>241</v>
@@ -3290,10 +3441,10 @@
         <v>143</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>350</v>
+        <v>382</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>351</v>
+        <v>383</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>241</v>
@@ -3340,10 +3491,10 @@
         <v>100</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>352</v>
+        <v>384</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>353</v>
+        <v>385</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>231</v>
@@ -3393,7 +3544,7 @@
         <v>104</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>354</v>
+        <v>386</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>240</v>
@@ -3440,10 +3591,10 @@
         <v>146</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>355</v>
+        <v>387</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>356</v>
+        <v>388</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>270</v>
@@ -3490,10 +3641,10 @@
         <v>168</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>357</v>
+        <v>389</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>358</v>
+        <v>390</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>251</v>
@@ -3540,10 +3691,10 @@
         <v>83</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>359</v>
+        <v>391</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>360</v>
+        <v>392</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>231</v>
@@ -3593,7 +3744,7 @@
         <v>77</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>361</v>
+        <v>393</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>231</v>
@@ -3643,7 +3794,7 @@
         <v>109</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>362</v>
+        <v>394</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>231</v>
@@ -3690,10 +3841,10 @@
         <v>204</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>363</v>
+        <v>395</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>364</v>
+        <v>396</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>231</v>
@@ -3740,10 +3891,10 @@
         <v>206</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>365</v>
+        <v>397</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>366</v>
+        <v>398</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>295</v>
@@ -3790,10 +3941,10 @@
         <v>118</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>367</v>
+        <v>399</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>368</v>
+        <v>400</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>231</v>
@@ -3843,7 +3994,7 @@
         <v>112</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>369</v>
+        <v>401</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>245</v>
@@ -3890,10 +4041,10 @@
         <v>207</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>370</v>
+        <v>402</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>371</v>
+        <v>403</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>270</v>
@@ -3940,10 +4091,10 @@
         <v>169</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>372</v>
+        <v>404</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>373</v>
+        <v>405</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>241</v>
@@ -3993,7 +4144,7 @@
         <v>89</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>374</v>
+        <v>406</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>296</v>
@@ -4040,10 +4191,10 @@
         <v>145</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>375</v>
+        <v>407</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>376</v>
+        <v>408</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>231</v>
@@ -4093,7 +4244,7 @@
         <v>71</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>377</v>
+        <v>409</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>230</v>
@@ -4140,10 +4291,10 @@
         <v>161</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>378</v>
+        <v>410</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>379</v>
+        <v>411</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>241</v>
@@ -4190,10 +4341,10 @@
         <v>114</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>380</v>
+        <v>412</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>381</v>
+        <v>413</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>236</v>
@@ -4243,7 +4394,7 @@
         <v>116</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>382</v>
+        <v>414</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>250</v>
@@ -4293,7 +4444,7 @@
         <v>90</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>383</v>
+        <v>415</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>296</v>
@@ -4340,10 +4491,10 @@
         <v>159</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>384</v>
+        <v>416</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>385</v>
+        <v>417</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>247</v>
@@ -4390,10 +4541,10 @@
         <v>172</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>386</v>
+        <v>418</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>387</v>
+        <v>419</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>300</v>
@@ -4440,10 +4591,10 @@
         <v>126</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>388</v>
+        <v>420</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>389</v>
+        <v>421</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>250</v>
@@ -4490,10 +4641,10 @@
         <v>92</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>390</v>
+        <v>422</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>391</v>
+        <v>423</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>236</v>
@@ -4540,10 +4691,10 @@
         <v>208</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>392</v>
+        <v>424</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>393</v>
+        <v>425</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>250</v>
@@ -4590,10 +4741,10 @@
         <v>86</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>394</v>
+        <v>426</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>395</v>
+        <v>427</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>231</v>
@@ -4640,10 +4791,10 @@
         <v>148</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>396</v>
+        <v>428</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>397</v>
+        <v>429</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>241</v>
@@ -4690,10 +4841,10 @@
         <v>103</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>398</v>
+        <v>430</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>399</v>
+        <v>431</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>231</v>
@@ -4743,7 +4894,7 @@
         <v>80</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>400</v>
+        <v>432</v>
       </c>
       <c r="D32" s="10" t="s">
         <v>231</v>
@@ -4790,10 +4941,10 @@
         <v>144</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>401</v>
+        <v>433</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>402</v>
+        <v>434</v>
       </c>
       <c r="D33" s="10" t="s">
         <v>296</v>
@@ -4840,10 +4991,10 @@
         <v>209</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>403</v>
+        <v>435</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>404</v>
+        <v>436</v>
       </c>
       <c r="D34" s="10" t="s">
         <v>236</v>
@@ -4890,10 +5041,10 @@
         <v>74</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>405</v>
+        <v>437</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>406</v>
+        <v>438</v>
       </c>
       <c r="D35" s="10" t="s">
         <v>231</v>
@@ -4940,10 +5091,10 @@
         <v>120</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>407</v>
+        <v>439</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>408</v>
+        <v>440</v>
       </c>
       <c r="D36" s="10" t="s">
         <v>231</v>
@@ -4993,7 +5144,7 @@
         <v>173</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>409</v>
+        <v>441</v>
       </c>
       <c r="D37" s="10" t="s">
         <v>276</v>
@@ -5040,10 +5191,10 @@
         <v>129</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>410</v>
+        <v>442</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>411</v>
+        <v>443</v>
       </c>
       <c r="D38" s="10" t="s">
         <v>230</v>
@@ -5090,10 +5241,10 @@
         <v>174</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>412</v>
+        <v>444</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>413</v>
+        <v>445</v>
       </c>
       <c r="D39" s="10" t="s">
         <v>231</v>
@@ -5140,10 +5291,10 @@
         <v>210</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>414</v>
+        <v>446</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>415</v>
+        <v>447</v>
       </c>
       <c r="D40" s="10" t="s">
         <v>230</v>
@@ -5190,10 +5341,10 @@
         <v>131</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>416</v>
+        <v>448</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>417</v>
+        <v>449</v>
       </c>
       <c r="D41" s="10" t="s">
         <v>231</v>
@@ -5240,10 +5391,10 @@
         <v>132</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>418</v>
+        <v>450</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>419</v>
+        <v>451</v>
       </c>
       <c r="D42" s="10" t="s">
         <v>231</v>
@@ -5290,10 +5441,10 @@
         <v>107</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>420</v>
+        <v>452</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>421</v>
+        <v>453</v>
       </c>
       <c r="D43" s="10" t="s">
         <v>236</v>
@@ -5340,10 +5491,10 @@
         <v>211</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>422</v>
+        <v>454</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>423</v>
+        <v>455</v>
       </c>
       <c r="D44" s="10" t="s">
         <v>301</v>
@@ -5390,10 +5541,10 @@
         <v>213</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>424</v>
+        <v>456</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>425</v>
+        <v>457</v>
       </c>
       <c r="D45" s="10" t="s">
         <v>230</v>
@@ -5440,10 +5591,10 @@
         <v>124</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>426</v>
+        <v>458</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>427</v>
+        <v>459</v>
       </c>
       <c r="D46" s="10" t="s">
         <v>230</v>
@@ -5490,10 +5641,10 @@
         <v>134</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>428</v>
+        <v>460</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>429</v>
+        <v>461</v>
       </c>
       <c r="D47" s="10" t="s">
         <v>277</v>
@@ -5540,10 +5691,10 @@
         <v>163</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>430</v>
+        <v>462</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>431</v>
+        <v>463</v>
       </c>
       <c r="D48" s="10" t="s">
         <v>252</v>
@@ -5593,7 +5744,7 @@
         <v>155</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>432</v>
+        <v>464</v>
       </c>
       <c r="D49" s="10" t="s">
         <v>231</v>
@@ -5643,7 +5794,7 @@
         <v>158</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>433</v>
+        <v>465</v>
       </c>
       <c r="D50" s="10" t="s">
         <v>296</v>
@@ -5690,10 +5841,10 @@
         <v>136</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>434</v>
+        <v>466</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>435</v>
+        <v>467</v>
       </c>
       <c r="D51" s="10" t="s">
         <v>246</v>
@@ -5740,10 +5891,10 @@
         <v>215</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>436</v>
+        <v>468</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>437</v>
+        <v>469</v>
       </c>
       <c r="D52" s="10" t="s">
         <v>278</v>
@@ -5790,10 +5941,10 @@
         <v>139</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>438</v>
+        <v>470</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>439</v>
+        <v>471</v>
       </c>
       <c r="D53" s="10" t="s">
         <v>302</v>
@@ -5843,7 +5994,7 @@
         <v>110</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>440</v>
+        <v>472</v>
       </c>
       <c r="D54" s="10" t="s">
         <v>241</v>
@@ -5890,10 +6041,10 @@
         <v>175</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>441</v>
+        <v>473</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>442</v>
+        <v>474</v>
       </c>
       <c r="D55" s="10" t="s">
         <v>231</v>
@@ -5940,10 +6091,10 @@
         <v>141</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>443</v>
+        <v>475</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>444</v>
+        <v>476</v>
       </c>
       <c r="D56" s="10" t="s">
         <v>241</v>
@@ -5990,10 +6141,10 @@
         <v>178</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>445</v>
+        <v>477</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>446</v>
+        <v>478</v>
       </c>
       <c r="D57" s="10" t="s">
         <v>230</v>
@@ -6040,10 +6191,10 @@
         <v>149</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>447</v>
+        <v>479</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>448</v>
+        <v>480</v>
       </c>
       <c r="D58" s="10" t="s">
         <v>241</v>
@@ -6090,10 +6241,10 @@
         <v>217</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>449</v>
+        <v>481</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>450</v>
+        <v>482</v>
       </c>
       <c r="D59" s="10" t="s">
         <v>301</v>
@@ -6140,10 +6291,10 @@
         <v>180</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>451</v>
+        <v>483</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>452</v>
+        <v>484</v>
       </c>
       <c r="D60" s="10" t="s">
         <v>230</v>
@@ -6190,10 +6341,10 @@
         <v>94</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>453</v>
+        <v>485</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>454</v>
+        <v>486</v>
       </c>
       <c r="D61" s="10" t="s">
         <v>230</v>
@@ -6240,10 +6391,10 @@
         <v>164</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>455</v>
+        <v>487</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>456</v>
+        <v>488</v>
       </c>
       <c r="D62" s="10" t="s">
         <v>248</v>
@@ -6290,10 +6441,10 @@
         <v>183</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>457</v>
+        <v>489</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>458</v>
+        <v>490</v>
       </c>
       <c r="D63" s="10" t="s">
         <v>247</v>
@@ -6340,10 +6491,10 @@
         <v>97</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>459</v>
+        <v>491</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>460</v>
+        <v>492</v>
       </c>
       <c r="D64" s="10" t="s">
         <v>231</v>
@@ -6390,10 +6541,10 @@
         <v>185</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>461</v>
+        <v>493</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>462</v>
+        <v>494</v>
       </c>
       <c r="D65" s="10" t="s">
         <v>250</v>
@@ -6440,10 +6591,10 @@
         <v>187</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>463</v>
+        <v>495</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>421</v>
+        <v>453</v>
       </c>
       <c r="D66" s="10" t="s">
         <v>236</v>
@@ -6493,7 +6644,7 @@
         <v>219</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>464</v>
+        <v>496</v>
       </c>
       <c r="D67" s="10" t="s">
         <v>295</v>
@@ -6540,10 +6691,10 @@
         <v>190</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>465</v>
+        <v>497</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>466</v>
+        <v>498</v>
       </c>
       <c r="D68" s="10" t="s">
         <v>251</v>
@@ -6590,10 +6741,10 @@
         <v>193</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>467</v>
+        <v>499</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>468</v>
+        <v>500</v>
       </c>
       <c r="D69" s="10" t="s">
         <v>252</v>
@@ -6640,10 +6791,10 @@
         <v>151</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>447</v>
+        <v>479</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>469</v>
+        <v>501</v>
       </c>
       <c r="D70" s="10" t="s">
         <v>241</v>
@@ -6690,10 +6841,10 @@
         <v>167</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>470</v>
+        <v>502</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>471</v>
+        <v>503</v>
       </c>
       <c r="D71" s="10" t="s">
         <v>231</v>
@@ -6740,10 +6891,10 @@
         <v>121</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>472</v>
+        <v>504</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>473</v>
+        <v>505</v>
       </c>
       <c r="D72" s="10" t="s">
         <v>236</v>
@@ -6790,10 +6941,10 @@
         <v>197</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>474</v>
+        <v>506</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>475</v>
+        <v>507</v>
       </c>
       <c r="D73" s="10" t="s">
         <v>252</v>
@@ -6840,10 +6991,10 @@
         <v>195</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>476</v>
+        <v>508</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>477</v>
+        <v>509</v>
       </c>
       <c r="D74" s="10" t="s">
         <v>252</v>
@@ -6890,10 +7041,10 @@
         <v>200</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>478</v>
+        <v>510</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>479</v>
+        <v>511</v>
       </c>
       <c r="D75" s="10" t="s">
         <v>231</v>
@@ -6943,7 +7094,7 @@
         <v>152</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>480</v>
+        <v>512</v>
       </c>
       <c r="D76" s="10" t="s">
         <v>296</v>
@@ -6993,7 +7144,7 @@
         <v>305</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>481</v>
+        <v>513</v>
       </c>
       <c r="D77" s="10" t="s">
         <v>296</v>
@@ -7036,10 +7187,10 @@
         <v>281</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>482</v>
+        <v>514</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>483</v>
+        <v>515</v>
       </c>
       <c r="D78" s="10" t="s">
         <v>270</v>
@@ -7085,7 +7236,7 @@
         <v>306</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>484</v>
+        <v>516</v>
       </c>
       <c r="D79" s="10" t="s">
         <v>296</v>
@@ -7128,10 +7279,10 @@
         <v>283</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>485</v>
+        <v>517</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>486</v>
+        <v>518</v>
       </c>
       <c r="D80" s="10" t="s">
         <v>276</v>
@@ -7174,10 +7325,10 @@
         <v>307</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>487</v>
+        <v>519</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>488</v>
+        <v>520</v>
       </c>
       <c r="D81" s="10" t="s">
         <v>308</v>
@@ -7220,10 +7371,10 @@
         <v>284</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>489</v>
+        <v>521</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>490</v>
+        <v>522</v>
       </c>
       <c r="D82" s="10" t="s">
         <v>285</v>
@@ -7269,7 +7420,7 @@
         <v>309</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>491</v>
+        <v>523</v>
       </c>
       <c r="D83" s="10" t="s">
         <v>310</v>
@@ -7312,10 +7463,10 @@
         <v>286</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>492</v>
+        <v>524</v>
       </c>
       <c r="C84" s="10" t="s">
-        <v>493</v>
+        <v>525</v>
       </c>
       <c r="D84" s="10" t="s">
         <v>248</v>
@@ -7358,10 +7509,10 @@
         <v>311</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>494</v>
+        <v>526</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>495</v>
+        <v>527</v>
       </c>
       <c r="D85" s="10" t="s">
         <v>300</v>
@@ -7404,10 +7555,10 @@
         <v>287</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>496</v>
+        <v>528</v>
       </c>
       <c r="C86" s="10" t="s">
-        <v>497</v>
+        <v>529</v>
       </c>
       <c r="D86" s="10" t="s">
         <v>230</v>
@@ -7450,10 +7601,10 @@
         <v>312</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>498</v>
+        <v>530</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>499</v>
+        <v>531</v>
       </c>
       <c r="D87" s="10" t="s">
         <v>313</v>
@@ -7496,10 +7647,10 @@
         <v>314</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>500</v>
+        <v>532</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>501</v>
+        <v>533</v>
       </c>
       <c r="D88" s="10" t="s">
         <v>240</v>
@@ -7542,10 +7693,10 @@
         <v>315</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>502</v>
+        <v>534</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>503</v>
+        <v>535</v>
       </c>
       <c r="D89" s="10" t="s">
         <v>296</v>
@@ -7588,10 +7739,10 @@
         <v>152</v>
       </c>
       <c r="B90" s="10" t="s">
-        <v>504</v>
+        <v>536</v>
       </c>
       <c r="C90" s="10" t="s">
-        <v>505</v>
+        <v>537</v>
       </c>
       <c r="D90" s="10" t="s">
         <v>296</v>
@@ -7634,10 +7785,10 @@
         <v>288</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>506</v>
+        <v>538</v>
       </c>
       <c r="C91" s="10" t="s">
-        <v>507</v>
+        <v>539</v>
       </c>
       <c r="D91" s="10" t="s">
         <v>276</v>
@@ -7680,10 +7831,10 @@
         <v>316</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>508</v>
+        <v>540</v>
       </c>
       <c r="C92" s="10" t="s">
-        <v>509</v>
+        <v>541</v>
       </c>
       <c r="D92" s="10" t="s">
         <v>296</v>
@@ -7726,10 +7877,10 @@
         <v>317</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>510</v>
+        <v>542</v>
       </c>
       <c r="C93" s="10" t="s">
-        <v>511</v>
+        <v>543</v>
       </c>
       <c r="D93" s="10" t="s">
         <v>313</v>
@@ -7772,10 +7923,10 @@
         <v>318</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>512</v>
+        <v>544</v>
       </c>
       <c r="C94" s="10" t="s">
-        <v>513</v>
+        <v>545</v>
       </c>
       <c r="D94" s="10" t="s">
         <v>319</v>
@@ -7818,10 +7969,10 @@
         <v>320</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>514</v>
+        <v>546</v>
       </c>
       <c r="C95" s="10" t="s">
-        <v>515</v>
+        <v>547</v>
       </c>
       <c r="D95" s="10" t="s">
         <v>296</v>
@@ -7864,10 +8015,10 @@
         <v>289</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>516</v>
+        <v>548</v>
       </c>
       <c r="C96" s="10" t="s">
-        <v>517</v>
+        <v>549</v>
       </c>
       <c r="D96" s="10" t="s">
         <v>236</v>
@@ -7910,10 +8061,10 @@
         <v>321</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>518</v>
+        <v>550</v>
       </c>
       <c r="C97" s="10" t="s">
-        <v>519</v>
+        <v>551</v>
       </c>
       <c r="D97" s="10" t="s">
         <v>230</v>
@@ -7956,10 +8107,10 @@
         <v>290</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>520</v>
+        <v>552</v>
       </c>
       <c r="C98" s="10" t="s">
-        <v>521</v>
+        <v>553</v>
       </c>
       <c r="D98" s="10" t="s">
         <v>252</v>
@@ -8002,10 +8153,10 @@
         <v>291</v>
       </c>
       <c r="B99" s="10" t="s">
-        <v>522</v>
+        <v>554</v>
       </c>
       <c r="C99" s="10" t="s">
-        <v>523</v>
+        <v>555</v>
       </c>
       <c r="D99" s="10" t="s">
         <v>236</v>
@@ -8048,10 +8199,10 @@
         <v>322</v>
       </c>
       <c r="B100" s="10" t="s">
-        <v>524</v>
+        <v>556</v>
       </c>
       <c r="C100" s="10" t="s">
-        <v>525</v>
+        <v>557</v>
       </c>
       <c r="D100" s="10" t="s">
         <v>296</v>
@@ -8094,10 +8245,10 @@
         <v>292</v>
       </c>
       <c r="B101" s="10" t="s">
-        <v>526</v>
+        <v>558</v>
       </c>
       <c r="C101" s="10" t="s">
-        <v>527</v>
+        <v>559</v>
       </c>
       <c r="D101" s="10" t="s">
         <v>231</v>
@@ -8140,10 +8291,10 @@
         <v>293</v>
       </c>
       <c r="B102" s="10" t="s">
-        <v>528</v>
+        <v>560</v>
       </c>
       <c r="C102" s="10" t="s">
-        <v>529</v>
+        <v>561</v>
       </c>
       <c r="D102" s="10" t="s">
         <v>251</v>
@@ -8186,10 +8337,10 @@
         <v>323</v>
       </c>
       <c r="B103" s="10" t="s">
-        <v>530</v>
+        <v>562</v>
       </c>
       <c r="C103" s="10" t="s">
-        <v>531</v>
+        <v>563</v>
       </c>
       <c r="D103" s="10" t="s">
         <v>324</v>
@@ -8232,10 +8383,10 @@
         <v>325</v>
       </c>
       <c r="B104" s="10" t="s">
-        <v>532</v>
+        <v>564</v>
       </c>
       <c r="C104" s="10" t="s">
-        <v>533</v>
+        <v>565</v>
       </c>
       <c r="D104" s="10" t="s">
         <v>308</v>
@@ -8278,10 +8429,10 @@
         <v>326</v>
       </c>
       <c r="B105" s="10" t="s">
-        <v>534</v>
+        <v>566</v>
       </c>
       <c r="C105" s="10" t="s">
-        <v>535</v>
+        <v>567</v>
       </c>
       <c r="D105" s="10" t="s">
         <v>302</v>
@@ -8324,10 +8475,10 @@
         <v>327</v>
       </c>
       <c r="B106" s="10" t="s">
-        <v>536</v>
+        <v>568</v>
       </c>
       <c r="C106" s="10" t="s">
-        <v>537</v>
+        <v>569</v>
       </c>
       <c r="D106" s="10" t="s">
         <v>240</v>
@@ -8370,10 +8521,10 @@
         <v>328</v>
       </c>
       <c r="B107" s="10" t="s">
-        <v>538</v>
+        <v>570</v>
       </c>
       <c r="C107" s="10" t="s">
-        <v>539</v>
+        <v>571</v>
       </c>
       <c r="D107" s="10" t="s">
         <v>329</v>
@@ -8416,10 +8567,10 @@
         <v>330</v>
       </c>
       <c r="B108" s="10" t="s">
-        <v>540</v>
+        <v>572</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>541</v>
+        <v>573</v>
       </c>
       <c r="D108" s="10" t="s">
         <v>246</v>
@@ -8473,7 +8624,7 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="29" t="s">
-        <v>542</v>
+        <v>574</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -8483,208 +8634,208 @@
       <c r="H2" s="29"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="50" t="s">
-        <v>543</v>
-      </c>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
+      <c r="B4" s="61" t="s">
+        <v>575</v>
+      </c>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="61"/>
+      <c r="I4" s="61"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="51" t="s">
-        <v>544</v>
-      </c>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="51"/>
-      <c r="H5" s="51"/>
-      <c r="I5" s="51"/>
+      <c r="B5" s="62" t="s">
+        <v>576</v>
+      </c>
+      <c r="C5" s="62"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="62"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="51" t="s">
-        <v>545</v>
-      </c>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
+      <c r="B6" s="62" t="s">
+        <v>577</v>
+      </c>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
+      <c r="H6" s="62"/>
+      <c r="I6" s="62"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="51" t="s">
+      <c r="B7" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="51"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
-      <c r="G7" s="51"/>
-      <c r="H7" s="51"/>
-      <c r="I7" s="51"/>
+      <c r="C7" s="62"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="62"/>
+      <c r="I7" s="62"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B8" s="51" t="s">
-        <v>546</v>
-      </c>
-      <c r="C8" s="51"/>
-      <c r="D8" s="51"/>
-      <c r="E8" s="51"/>
-      <c r="F8" s="51"/>
-      <c r="G8" s="51"/>
-      <c r="H8" s="51"/>
-      <c r="I8" s="51"/>
+      <c r="B8" s="62" t="s">
+        <v>578</v>
+      </c>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="62"/>
+      <c r="H8" s="62"/>
+      <c r="I8" s="62"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="51" t="s">
-        <v>547</v>
-      </c>
-      <c r="C9" s="51"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="51"/>
-      <c r="G9" s="51"/>
-      <c r="H9" s="51"/>
-      <c r="I9" s="51"/>
+      <c r="B9" s="62" t="s">
+        <v>579</v>
+      </c>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="62"/>
+      <c r="G9" s="62"/>
+      <c r="H9" s="62"/>
+      <c r="I9" s="62"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="51" t="s">
+      <c r="B10" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="51"/>
-      <c r="D10" s="51"/>
-      <c r="E10" s="51"/>
-      <c r="F10" s="51"/>
-      <c r="G10" s="51"/>
-      <c r="H10" s="51"/>
-      <c r="I10" s="51"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="50" t="s">
-        <v>548</v>
-      </c>
-      <c r="C11" s="50"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="50"/>
+      <c r="B11" s="61" t="s">
+        <v>580</v>
+      </c>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="51" t="s">
-        <v>549</v>
-      </c>
-      <c r="C12" s="51"/>
-      <c r="D12" s="51"/>
-      <c r="E12" s="51"/>
-      <c r="F12" s="51"/>
-      <c r="G12" s="51"/>
-      <c r="H12" s="51"/>
-      <c r="I12" s="51"/>
+      <c r="B12" s="62" t="s">
+        <v>581</v>
+      </c>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="62"/>
+      <c r="I12" s="62"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="51" t="s">
-        <v>550</v>
-      </c>
-      <c r="C13" s="51"/>
-      <c r="D13" s="51"/>
-      <c r="E13" s="51"/>
-      <c r="F13" s="51"/>
-      <c r="G13" s="51"/>
-      <c r="H13" s="51"/>
-      <c r="I13" s="51"/>
+      <c r="B13" s="62" t="s">
+        <v>582</v>
+      </c>
+      <c r="C13" s="62"/>
+      <c r="D13" s="62"/>
+      <c r="E13" s="62"/>
+      <c r="F13" s="62"/>
+      <c r="G13" s="62"/>
+      <c r="H13" s="62"/>
+      <c r="I13" s="62"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="51" t="s">
-        <v>551</v>
-      </c>
-      <c r="C14" s="51"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="51"/>
-      <c r="F14" s="51"/>
-      <c r="G14" s="51"/>
-      <c r="H14" s="51"/>
-      <c r="I14" s="51"/>
+      <c r="B14" s="62" t="s">
+        <v>583</v>
+      </c>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
+      <c r="G14" s="62"/>
+      <c r="H14" s="62"/>
+      <c r="I14" s="62"/>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="51" t="s">
-        <v>552</v>
-      </c>
-      <c r="C15" s="51"/>
-      <c r="D15" s="51"/>
-      <c r="E15" s="51"/>
-      <c r="F15" s="51"/>
-      <c r="G15" s="51"/>
-      <c r="H15" s="51"/>
-      <c r="I15" s="51"/>
+      <c r="B15" s="62" t="s">
+        <v>584</v>
+      </c>
+      <c r="C15" s="62"/>
+      <c r="D15" s="62"/>
+      <c r="E15" s="62"/>
+      <c r="F15" s="62"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="62"/>
+      <c r="I15" s="62"/>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="51" t="s">
-        <v>553</v>
-      </c>
-      <c r="C16" s="51"/>
-      <c r="D16" s="51"/>
-      <c r="E16" s="51"/>
-      <c r="F16" s="51"/>
-      <c r="G16" s="51"/>
-      <c r="H16" s="51"/>
-      <c r="I16" s="51"/>
+      <c r="B16" s="62" t="s">
+        <v>585</v>
+      </c>
+      <c r="C16" s="62"/>
+      <c r="D16" s="62"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="62"/>
+      <c r="G16" s="62"/>
+      <c r="H16" s="62"/>
+      <c r="I16" s="62"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="51" t="s">
-        <v>554</v>
-      </c>
-      <c r="C17" s="51"/>
-      <c r="D17" s="51"/>
-      <c r="E17" s="51"/>
-      <c r="F17" s="51"/>
-      <c r="G17" s="51"/>
-      <c r="H17" s="51"/>
-      <c r="I17" s="51"/>
+      <c r="B17" s="62" t="s">
+        <v>586</v>
+      </c>
+      <c r="C17" s="62"/>
+      <c r="D17" s="62"/>
+      <c r="E17" s="62"/>
+      <c r="F17" s="62"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="62"/>
+      <c r="I17" s="62"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="51" t="s">
-        <v>555</v>
-      </c>
-      <c r="C18" s="51"/>
-      <c r="D18" s="51"/>
-      <c r="E18" s="51"/>
-      <c r="F18" s="51"/>
-      <c r="G18" s="51"/>
-      <c r="H18" s="51"/>
-      <c r="I18" s="51"/>
+      <c r="B18" s="62" t="s">
+        <v>587</v>
+      </c>
+      <c r="C18" s="62"/>
+      <c r="D18" s="62"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="62"/>
+      <c r="G18" s="62"/>
+      <c r="H18" s="62"/>
+      <c r="I18" s="62"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="51" t="s">
-        <v>556</v>
-      </c>
-      <c r="C19" s="51"/>
-      <c r="D19" s="51"/>
-      <c r="E19" s="51"/>
-      <c r="F19" s="51"/>
-      <c r="G19" s="51"/>
-      <c r="H19" s="51"/>
-      <c r="I19" s="51"/>
+      <c r="B19" s="62" t="s">
+        <v>588</v>
+      </c>
+      <c r="C19" s="62"/>
+      <c r="D19" s="62"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
+      <c r="G19" s="62"/>
+      <c r="H19" s="62"/>
+      <c r="I19" s="62"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="51" t="s">
-        <v>557</v>
-      </c>
-      <c r="C20" s="51"/>
-      <c r="D20" s="51"/>
-      <c r="E20" s="51"/>
-      <c r="F20" s="51"/>
-      <c r="G20" s="51"/>
-      <c r="H20" s="51"/>
-      <c r="I20" s="51"/>
+      <c r="B20" s="62" t="s">
+        <v>589</v>
+      </c>
+      <c r="C20" s="62"/>
+      <c r="D20" s="62"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
+      <c r="G20" s="62"/>
+      <c r="H20" s="62"/>
+      <c r="I20" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -18293,13 +18444,18 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:I7"/>
+  <dimension ref="B2:I109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="5" width="14" customWidth="1"/>
+    <col min="6" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="29" t="s">
         <v>332</v>
       </c>
@@ -18309,88 +18465,1902 @@
       <c r="F2" s="29"/>
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="50" t="s">
+        <v>333</v>
+      </c>
+      <c r="C3" s="50"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="6">
+        <v>75</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6">
+        <v>2</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6">
+        <v>14</v>
+      </c>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6">
+        <v>16</v>
+      </c>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="51" t="s">
+        <v>338</v>
+      </c>
+      <c r="C10" s="51"/>
+      <c r="D10" s="51"/>
+      <c r="E10" s="51"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="51"/>
+      <c r="H10" s="51"/>
+      <c r="I10" s="51"/>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>342</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="C13" s="46">
+        <v>4</v>
+      </c>
+      <c r="D13" s="46">
+        <v>0</v>
+      </c>
+      <c r="E13" s="52">
+        <v>4</v>
+      </c>
+      <c r="F13" s="53" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="10" t="s">
+        <v>345</v>
+      </c>
+      <c r="C14" s="46">
+        <v>3</v>
+      </c>
+      <c r="D14" s="46">
+        <v>3</v>
+      </c>
+      <c r="E14" s="52">
+        <v>6</v>
+      </c>
+      <c r="F14" s="54" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="10" t="s">
+        <v>347</v>
+      </c>
+      <c r="C15" s="46">
+        <v>9</v>
+      </c>
+      <c r="D15" s="46">
+        <v>3</v>
+      </c>
+      <c r="E15" s="52">
+        <v>12</v>
+      </c>
+      <c r="F15" s="54" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="10" t="s">
+        <v>349</v>
+      </c>
+      <c r="C16" s="46">
+        <v>8</v>
+      </c>
+      <c r="D16" s="46">
+        <v>8</v>
+      </c>
+      <c r="E16" s="52">
+        <v>16</v>
+      </c>
+      <c r="F16" s="54" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="10" t="s">
+        <v>351</v>
+      </c>
+      <c r="C17" s="46">
+        <v>3</v>
+      </c>
+      <c r="D17" s="46">
+        <v>5</v>
+      </c>
+      <c r="E17" s="52">
+        <v>8</v>
+      </c>
+      <c r="F17" s="55" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C18" s="46">
+        <v>0</v>
+      </c>
+      <c r="D18" s="46">
+        <v>6</v>
+      </c>
+      <c r="E18" s="52">
+        <v>6</v>
+      </c>
+      <c r="F18" s="55" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="C19" s="46">
+        <v>4</v>
+      </c>
+      <c r="D19" s="46">
+        <v>3</v>
+      </c>
+      <c r="E19" s="52">
+        <v>7</v>
+      </c>
+      <c r="F19" s="54" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="C20" s="46">
+        <v>7</v>
+      </c>
+      <c r="D20" s="46">
+        <v>7</v>
+      </c>
+      <c r="E20" s="52">
+        <v>14</v>
+      </c>
+      <c r="F20" s="54" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="C21" s="46">
+        <v>1</v>
+      </c>
+      <c r="D21" s="46">
+        <v>1</v>
+      </c>
+      <c r="E21" s="52">
+        <v>2</v>
+      </c>
+      <c r="F21" s="55" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="56" t="s">
+        <v>361</v>
+      </c>
+      <c r="C22" s="57">
+        <v>39</v>
+      </c>
+      <c r="D22" s="57">
+        <v>36</v>
+      </c>
+      <c r="E22" s="57">
+        <v>75</v>
+      </c>
+      <c r="F22" s="58" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="59" t="s">
+        <v>362</v>
+      </c>
+      <c r="C25" s="59"/>
+      <c r="D25" s="59"/>
+      <c r="E25" s="59"/>
+      <c r="F25" s="59"/>
+      <c r="G25" s="59"/>
+      <c r="H25" s="59"/>
+      <c r="I25" s="59"/>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B27" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C27" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D27" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E27" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F27" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G27" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H27" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I27" s="9" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="10" t="s">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C28" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="D6" s="49" t="s">
+      <c r="D28" s="49" t="s">
         <v>251</v>
       </c>
-      <c r="E6" s="49" t="s">
+      <c r="E28" s="49" t="s">
         <v>84</v>
       </c>
-      <c r="F6" s="46">
-        <v>1</v>
-      </c>
-      <c r="G6" s="46">
-        <v>1</v>
-      </c>
-      <c r="H6" s="47">
+      <c r="F28" s="46">
+        <v>1</v>
+      </c>
+      <c r="G28" s="46">
+        <v>1</v>
+      </c>
+      <c r="H28" s="47">
         <v>675</v>
       </c>
-      <c r="I6" s="49" t="s">
+      <c r="I28" s="49" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="10" t="s">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C29" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="D7" s="49" t="s">
+      <c r="D29" s="49" t="s">
         <v>241</v>
       </c>
-      <c r="E7" s="49" t="s">
+      <c r="E29" s="49" t="s">
         <v>101</v>
       </c>
-      <c r="F7" s="46">
-        <v>1</v>
-      </c>
-      <c r="G7" s="46">
-        <v>1</v>
-      </c>
-      <c r="H7" s="47">
-        <v>0</v>
-      </c>
-      <c r="I7" s="49" t="s">
+      <c r="F29" s="46">
+        <v>1</v>
+      </c>
+      <c r="G29" s="46">
+        <v>1</v>
+      </c>
+      <c r="H29" s="47">
+        <v>0</v>
+      </c>
+      <c r="I29" s="49" t="s">
         <v>269</v>
       </c>
     </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B32" s="59" t="s">
+        <v>363</v>
+      </c>
+      <c r="C32" s="59"/>
+      <c r="D32" s="59"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="59"/>
+      <c r="H32" s="59"/>
+      <c r="I32" s="59"/>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B34" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B35" s="60" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="E35" s="46">
+        <v>1</v>
+      </c>
+      <c r="F35" s="46">
+        <v>1</v>
+      </c>
+      <c r="G35" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B36" s="60" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="E36" s="46">
+        <v>1</v>
+      </c>
+      <c r="F36" s="46">
+        <v>1</v>
+      </c>
+      <c r="G36" s="47">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B37" s="60" t="s">
+        <v>205</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="E37" s="46">
+        <v>1</v>
+      </c>
+      <c r="F37" s="46">
+        <v>1</v>
+      </c>
+      <c r="G37" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B38" s="60" t="s">
+        <v>82</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="E38" s="46">
+        <v>1</v>
+      </c>
+      <c r="F38" s="46">
+        <v>1</v>
+      </c>
+      <c r="G38" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B39" s="60" t="s">
+        <v>88</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="E39" s="46">
+        <v>1</v>
+      </c>
+      <c r="F39" s="46">
+        <v>1</v>
+      </c>
+      <c r="G39" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B40" s="60" t="s">
+        <v>127</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="E40" s="46">
+        <v>1</v>
+      </c>
+      <c r="F40" s="46">
+        <v>1</v>
+      </c>
+      <c r="G40" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B41" s="60" t="s">
+        <v>93</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="E41" s="46">
+        <v>2</v>
+      </c>
+      <c r="F41" s="46">
+        <v>10</v>
+      </c>
+      <c r="G41" s="47">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B42" s="60" t="s">
+        <v>93</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="E42" s="46">
+        <v>1</v>
+      </c>
+      <c r="F42" s="46">
+        <v>1</v>
+      </c>
+      <c r="G42" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B43" s="60" t="s">
+        <v>81</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="E43" s="46">
+        <v>3</v>
+      </c>
+      <c r="F43" s="46">
+        <v>7</v>
+      </c>
+      <c r="G43" s="47">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B44" s="60" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="E44" s="46">
+        <v>2</v>
+      </c>
+      <c r="F44" s="46">
+        <v>2</v>
+      </c>
+      <c r="G44" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B45" s="60" t="s">
+        <v>135</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="E45" s="46">
+        <v>1</v>
+      </c>
+      <c r="F45" s="46">
+        <v>1</v>
+      </c>
+      <c r="G45" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B46" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="E46" s="46">
+        <v>2</v>
+      </c>
+      <c r="F46" s="46">
+        <v>10</v>
+      </c>
+      <c r="G46" s="47">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B47" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="E47" s="46">
+        <v>1</v>
+      </c>
+      <c r="F47" s="46">
+        <v>1</v>
+      </c>
+      <c r="G47" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B48" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="E48" s="46">
+        <v>1</v>
+      </c>
+      <c r="F48" s="46">
+        <v>2</v>
+      </c>
+      <c r="G48" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B49" s="60" t="s">
+        <v>108</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E49" s="46">
+        <v>2</v>
+      </c>
+      <c r="F49" s="46">
+        <v>10</v>
+      </c>
+      <c r="G49" s="47">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B50" s="60" t="s">
+        <v>108</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E50" s="46">
+        <v>2</v>
+      </c>
+      <c r="F50" s="46">
+        <v>10</v>
+      </c>
+      <c r="G50" s="47">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B51" s="60" t="s">
+        <v>212</v>
+      </c>
+      <c r="C51" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="E51" s="46">
+        <v>1</v>
+      </c>
+      <c r="F51" s="46">
+        <v>1</v>
+      </c>
+      <c r="G51" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B52" s="60" t="s">
+        <v>214</v>
+      </c>
+      <c r="C52" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D52" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="E52" s="46">
+        <v>1</v>
+      </c>
+      <c r="F52" s="46">
+        <v>1</v>
+      </c>
+      <c r="G52" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B53" s="60" t="s">
+        <v>96</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="E53" s="46">
+        <v>2</v>
+      </c>
+      <c r="F53" s="46">
+        <v>10</v>
+      </c>
+      <c r="G53" s="47">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B54" s="60" t="s">
+        <v>156</v>
+      </c>
+      <c r="C54" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D54" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="E54" s="46">
+        <v>1</v>
+      </c>
+      <c r="F54" s="46">
+        <v>2</v>
+      </c>
+      <c r="G54" s="47">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B55" s="60" t="s">
+        <v>216</v>
+      </c>
+      <c r="C55" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="E55" s="46">
+        <v>1</v>
+      </c>
+      <c r="F55" s="46">
+        <v>2</v>
+      </c>
+      <c r="G55" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B56" s="60" t="s">
+        <v>140</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E56" s="46">
+        <v>2</v>
+      </c>
+      <c r="F56" s="46">
+        <v>10</v>
+      </c>
+      <c r="G56" s="47">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B57" s="60" t="s">
+        <v>176</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="E57" s="46">
+        <v>1</v>
+      </c>
+      <c r="F57" s="46">
+        <v>1</v>
+      </c>
+      <c r="G57" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B58" s="60" t="s">
+        <v>304</v>
+      </c>
+      <c r="C58" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D58" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="E58" s="46">
+        <v>3</v>
+      </c>
+      <c r="F58" s="46">
+        <v>9</v>
+      </c>
+      <c r="G58" s="47">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B59" s="60" t="s">
+        <v>106</v>
+      </c>
+      <c r="C59" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="E59" s="46">
+        <v>3</v>
+      </c>
+      <c r="F59" s="46">
+        <v>11</v>
+      </c>
+      <c r="G59" s="47">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B60" s="60" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="E60" s="46">
+        <v>3</v>
+      </c>
+      <c r="F60" s="46">
+        <v>5</v>
+      </c>
+      <c r="G60" s="47">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B61" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C61" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="E61" s="46">
+        <v>4</v>
+      </c>
+      <c r="F61" s="46">
+        <v>8</v>
+      </c>
+      <c r="G61" s="47">
+        <v>3725</v>
+      </c>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B62" s="60" t="s">
+        <v>218</v>
+      </c>
+      <c r="C62" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="E62" s="46">
+        <v>1</v>
+      </c>
+      <c r="F62" s="46">
+        <v>1</v>
+      </c>
+      <c r="G62" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B63" s="60" t="s">
+        <v>119</v>
+      </c>
+      <c r="C63" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D63" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="E63" s="46">
+        <v>4</v>
+      </c>
+      <c r="F63" s="46">
+        <v>4</v>
+      </c>
+      <c r="G63" s="47">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B64" s="60" t="s">
+        <v>95</v>
+      </c>
+      <c r="C64" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="E64" s="46">
+        <v>2</v>
+      </c>
+      <c r="F64" s="46">
+        <v>2</v>
+      </c>
+      <c r="G64" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B65" s="60" t="s">
+        <v>165</v>
+      </c>
+      <c r="C65" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="E65" s="46">
+        <v>1</v>
+      </c>
+      <c r="F65" s="46">
+        <v>2</v>
+      </c>
+      <c r="G65" s="47">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B66" s="60" t="s">
+        <v>184</v>
+      </c>
+      <c r="C66" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D66" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="E66" s="46">
+        <v>1</v>
+      </c>
+      <c r="F66" s="46">
+        <v>1</v>
+      </c>
+      <c r="G66" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B67" s="60" t="s">
+        <v>98</v>
+      </c>
+      <c r="C67" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D67" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="E67" s="46">
+        <v>4</v>
+      </c>
+      <c r="F67" s="46">
+        <v>18</v>
+      </c>
+      <c r="G67" s="47">
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B68" s="60" t="s">
+        <v>189</v>
+      </c>
+      <c r="C68" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D68" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E68" s="46">
+        <v>5</v>
+      </c>
+      <c r="F68" s="46">
+        <v>13</v>
+      </c>
+      <c r="G68" s="47">
+        <v>6075</v>
+      </c>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B69" s="60" t="s">
+        <v>189</v>
+      </c>
+      <c r="C69" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D69" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="E69" s="46">
+        <v>5</v>
+      </c>
+      <c r="F69" s="46">
+        <v>10</v>
+      </c>
+      <c r="G69" s="47">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B70" s="60" t="s">
+        <v>189</v>
+      </c>
+      <c r="C70" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D70" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="E70" s="46">
+        <v>2</v>
+      </c>
+      <c r="F70" s="46">
+        <v>2</v>
+      </c>
+      <c r="G70" s="47">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B71" s="60" t="s">
+        <v>249</v>
+      </c>
+      <c r="C71" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D71" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="E71" s="46">
+        <v>3</v>
+      </c>
+      <c r="F71" s="46">
+        <v>4</v>
+      </c>
+      <c r="G71" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B72" s="60" t="s">
+        <v>186</v>
+      </c>
+      <c r="C72" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D72" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="E72" s="46">
+        <v>1</v>
+      </c>
+      <c r="F72" s="46">
+        <v>1</v>
+      </c>
+      <c r="G72" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B73" s="60" t="s">
+        <v>188</v>
+      </c>
+      <c r="C73" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D73" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="E73" s="46">
+        <v>1</v>
+      </c>
+      <c r="F73" s="46">
+        <v>1</v>
+      </c>
+      <c r="G73" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B74" s="60" t="s">
+        <v>235</v>
+      </c>
+      <c r="C74" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D74" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="E74" s="46">
+        <v>7</v>
+      </c>
+      <c r="F74" s="46">
+        <v>35</v>
+      </c>
+      <c r="G74" s="47">
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B75" s="60" t="s">
+        <v>191</v>
+      </c>
+      <c r="C75" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D75" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="E75" s="46">
+        <v>2</v>
+      </c>
+      <c r="F75" s="46">
+        <v>2</v>
+      </c>
+      <c r="G75" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B76" s="60" t="s">
+        <v>191</v>
+      </c>
+      <c r="C76" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D76" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="E76" s="46">
+        <v>1</v>
+      </c>
+      <c r="F76" s="46">
+        <v>1</v>
+      </c>
+      <c r="G76" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B77" s="60" t="s">
+        <v>191</v>
+      </c>
+      <c r="C77" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D77" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="E77" s="46">
+        <v>1</v>
+      </c>
+      <c r="F77" s="46">
+        <v>1</v>
+      </c>
+      <c r="G77" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B78" s="60" t="s">
+        <v>299</v>
+      </c>
+      <c r="C78" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D78" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E78" s="46">
+        <v>11</v>
+      </c>
+      <c r="F78" s="46">
+        <v>25</v>
+      </c>
+      <c r="G78" s="47">
+        <v>10800</v>
+      </c>
+    </row>
+    <row r="79" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B79" s="60" t="s">
+        <v>237</v>
+      </c>
+      <c r="C79" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D79" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="E79" s="46">
+        <v>8</v>
+      </c>
+      <c r="F79" s="46">
+        <v>22</v>
+      </c>
+      <c r="G79" s="47">
+        <v>10800</v>
+      </c>
+    </row>
+    <row r="80" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B80" s="60" t="s">
+        <v>297</v>
+      </c>
+      <c r="C80" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D80" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="E80" s="46">
+        <v>4</v>
+      </c>
+      <c r="F80" s="46">
+        <v>23</v>
+      </c>
+      <c r="G80" s="47">
+        <v>12600</v>
+      </c>
+    </row>
+    <row r="81" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B81" s="60" t="s">
+        <v>194</v>
+      </c>
+      <c r="C81" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D81" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="E81" s="46">
+        <v>1</v>
+      </c>
+      <c r="F81" s="46">
+        <v>1</v>
+      </c>
+      <c r="G81" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="82" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B82" s="60" t="s">
+        <v>123</v>
+      </c>
+      <c r="C82" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D82" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="E82" s="46">
+        <v>4</v>
+      </c>
+      <c r="F82" s="46">
+        <v>5</v>
+      </c>
+      <c r="G82" s="47">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="83" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B83" s="60" t="s">
+        <v>123</v>
+      </c>
+      <c r="C83" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D83" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E83" s="46">
+        <v>6</v>
+      </c>
+      <c r="F83" s="46">
+        <v>12</v>
+      </c>
+      <c r="G83" s="47">
+        <v>7350</v>
+      </c>
+    </row>
+    <row r="84" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B84" s="60" t="s">
+        <v>150</v>
+      </c>
+      <c r="C84" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D84" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="E84" s="46">
+        <v>2</v>
+      </c>
+      <c r="F84" s="46">
+        <v>5</v>
+      </c>
+      <c r="G84" s="47">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="85" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B85" s="60" t="s">
+        <v>150</v>
+      </c>
+      <c r="C85" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D85" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="E85" s="46">
+        <v>1</v>
+      </c>
+      <c r="F85" s="46">
+        <v>4</v>
+      </c>
+      <c r="G85" s="47">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="86" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B86" s="60" t="s">
+        <v>303</v>
+      </c>
+      <c r="C86" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D86" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="E86" s="46">
+        <v>6</v>
+      </c>
+      <c r="F86" s="46">
+        <v>14</v>
+      </c>
+      <c r="G86" s="47">
+        <v>6600</v>
+      </c>
+    </row>
+    <row r="87" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B87" s="60" t="s">
+        <v>138</v>
+      </c>
+      <c r="C87" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D87" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="E87" s="46">
+        <v>2</v>
+      </c>
+      <c r="F87" s="46">
+        <v>4</v>
+      </c>
+      <c r="G87" s="47">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="88" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B88" s="60" t="s">
+        <v>280</v>
+      </c>
+      <c r="C88" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D88" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E88" s="46">
+        <v>2</v>
+      </c>
+      <c r="F88" s="46">
+        <v>2</v>
+      </c>
+      <c r="G88" s="47">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="89" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B89" s="60" t="s">
+        <v>202</v>
+      </c>
+      <c r="C89" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D89" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="E89" s="46">
+        <v>2</v>
+      </c>
+      <c r="F89" s="46">
+        <v>10</v>
+      </c>
+      <c r="G89" s="47">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="90" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B90" s="60" t="s">
+        <v>239</v>
+      </c>
+      <c r="C90" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D90" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="E90" s="46">
+        <v>3</v>
+      </c>
+      <c r="F90" s="46">
+        <v>18</v>
+      </c>
+      <c r="G90" s="47">
+        <v>9800</v>
+      </c>
+    </row>
+    <row r="91" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B91" s="60" t="s">
+        <v>238</v>
+      </c>
+      <c r="C91" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D91" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="E91" s="46">
+        <v>2</v>
+      </c>
+      <c r="F91" s="46">
+        <v>6</v>
+      </c>
+      <c r="G91" s="47">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="92" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B92" s="60" t="s">
+        <v>238</v>
+      </c>
+      <c r="C92" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D92" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E92" s="46">
+        <v>4</v>
+      </c>
+      <c r="F92" s="46">
+        <v>17</v>
+      </c>
+      <c r="G92" s="47">
+        <v>10200</v>
+      </c>
+    </row>
+    <row r="93" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B93" s="60" t="s">
+        <v>122</v>
+      </c>
+      <c r="C93" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D93" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="E93" s="46">
+        <v>2</v>
+      </c>
+      <c r="F93" s="46">
+        <v>10</v>
+      </c>
+      <c r="G93" s="47">
+        <v>5500</v>
+      </c>
+    </row>
+    <row r="94" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B94" s="60" t="s">
+        <v>198</v>
+      </c>
+      <c r="C94" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D94" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="E94" s="46">
+        <v>5</v>
+      </c>
+      <c r="F94" s="46">
+        <v>41</v>
+      </c>
+      <c r="G94" s="47">
+        <v>21900</v>
+      </c>
+    </row>
+    <row r="95" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B95" s="60" t="s">
+        <v>198</v>
+      </c>
+      <c r="C95" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D95" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="E95" s="46">
+        <v>1</v>
+      </c>
+      <c r="F95" s="46">
+        <v>1</v>
+      </c>
+      <c r="G95" s="47">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="96" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B96" s="60" t="s">
+        <v>196</v>
+      </c>
+      <c r="C96" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D96" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E96" s="46">
+        <v>1</v>
+      </c>
+      <c r="F96" s="46">
+        <v>1</v>
+      </c>
+      <c r="G96" s="47">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="97" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B97" s="60" t="s">
+        <v>275</v>
+      </c>
+      <c r="C97" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D97" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="E97" s="46">
+        <v>3</v>
+      </c>
+      <c r="F97" s="46">
+        <v>12</v>
+      </c>
+      <c r="G97" s="47">
+        <v>5500</v>
+      </c>
+    </row>
+    <row r="98" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B98" s="60" t="s">
+        <v>274</v>
+      </c>
+      <c r="C98" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D98" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="E98" s="46">
+        <v>6</v>
+      </c>
+      <c r="F98" s="46">
+        <v>12</v>
+      </c>
+      <c r="G98" s="47">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="99" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B99" s="60" t="s">
+        <v>201</v>
+      </c>
+      <c r="C99" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D99" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="E99" s="46">
+        <v>1</v>
+      </c>
+      <c r="F99" s="46">
+        <v>1</v>
+      </c>
+      <c r="G99" s="47">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="100" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B100" s="60" t="s">
+        <v>153</v>
+      </c>
+      <c r="C100" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D100" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="E100" s="46">
+        <v>8</v>
+      </c>
+      <c r="F100" s="46">
+        <v>19</v>
+      </c>
+      <c r="G100" s="47">
+        <v>9300</v>
+      </c>
+    </row>
+    <row r="101" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B101" s="60" t="s">
+        <v>153</v>
+      </c>
+      <c r="C101" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D101" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E101" s="46">
+        <v>8</v>
+      </c>
+      <c r="F101" s="46">
+        <v>64</v>
+      </c>
+      <c r="G101" s="47">
+        <v>37200</v>
+      </c>
+    </row>
+    <row r="102" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B102" s="60" t="s">
+        <v>153</v>
+      </c>
+      <c r="C102" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D102" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="E102" s="46">
+        <v>1</v>
+      </c>
+      <c r="F102" s="46">
+        <v>4</v>
+      </c>
+      <c r="G102" s="47">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="103" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B103" s="60" t="s">
+        <v>153</v>
+      </c>
+      <c r="C103" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D103" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E103" s="46">
+        <v>6</v>
+      </c>
+      <c r="F103" s="46">
+        <v>43</v>
+      </c>
+      <c r="G103" s="47">
+        <v>25050</v>
+      </c>
+    </row>
+    <row r="104" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B104" s="60" t="s">
+        <v>153</v>
+      </c>
+      <c r="C104" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D104" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="E104" s="46">
+        <v>6</v>
+      </c>
+      <c r="F104" s="46">
+        <v>24</v>
+      </c>
+      <c r="G104" s="47">
+        <v>12700</v>
+      </c>
+    </row>
+    <row r="105" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B105" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="C105" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="E105" s="46">
+        <v>4</v>
+      </c>
+      <c r="F105" s="46">
+        <v>17</v>
+      </c>
+      <c r="G105" s="47">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="106" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B106" s="60" t="s">
+        <v>273</v>
+      </c>
+      <c r="C106" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D106" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="E106" s="46">
+        <v>4</v>
+      </c>
+      <c r="F106" s="46">
+        <v>12</v>
+      </c>
+      <c r="G106" s="47">
+        <v>6655</v>
+      </c>
+    </row>
+    <row r="107" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B107" s="60" t="s">
+        <v>272</v>
+      </c>
+      <c r="C107" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D107" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="E107" s="46">
+        <v>4</v>
+      </c>
+      <c r="F107" s="46">
+        <v>7</v>
+      </c>
+      <c r="G107" s="47">
+        <v>5680</v>
+      </c>
+    </row>
+    <row r="108" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B108" s="60" t="s">
+        <v>272</v>
+      </c>
+      <c r="C108" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D108" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E108" s="46">
+        <v>16</v>
+      </c>
+      <c r="F108" s="46">
+        <v>45</v>
+      </c>
+      <c r="G108" s="47">
+        <v>22300</v>
+      </c>
+    </row>
+    <row r="109" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B109" s="60" t="s">
+        <v>234</v>
+      </c>
+      <c r="C109" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D109" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="E109" s="46">
+        <v>15</v>
+      </c>
+      <c r="F109" s="46">
+        <v>34</v>
+      </c>
+      <c r="G109" s="47">
+        <v>19200</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2:H2"/>
+  <mergeCells count="13">
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="B6:C7"/>
+    <mergeCell ref="D6:E7"/>
+    <mergeCell ref="F6:G7"/>
+    <mergeCell ref="H6:I7"/>
+    <mergeCell ref="B10:I10"/>
+    <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B32:I32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -18411,7 +20381,7 @@
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="29" t="s">
-        <v>333</v>
+        <v>365</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -18423,7 +20393,7 @@
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="8" t="s">
-        <v>334</v>
+        <v>366</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
@@ -18447,13 +20417,13 @@
         <v>9</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>335</v>
+        <v>367</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>62</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>336</v>
+        <v>368</v>
       </c>
       <c r="I5" s="9" t="s">
         <v>68</v>
@@ -18869,7 +20839,7 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="29" t="s">
-        <v>337</v>
+        <v>369</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -18892,7 +20862,7 @@
         <v>267</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>336</v>
+        <v>368</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>68</v>

</xml_diff>